<commit_message>
molj-09-04-25 - local save 2.0
</commit_message>
<xml_diff>
--- a/ASCal/mapping.xlsx
+++ b/ASCal/mapping.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dbneri\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d3a15bcb956f50ef/Documents/Visual Studio 2010/Projects/ASCal/ASCal/"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="6" documentId="11_BAFEF71822B0808C92284253D5B5B0600DF5EED8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C3E0CF90-8CD9-4DA5-846E-BEE7248043C2}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="12510" windowHeight="9570"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -5466,7 +5467,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -5567,7 +5568,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -5603,11 +5604,24 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -5893,40 +5907,40 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AN109"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="9.28515625" style="2" customWidth="1"/>
+    <col min="1" max="2" width="9.33203125" style="2" customWidth="1"/>
     <col min="3" max="3" width="12" style="2" customWidth="1"/>
-    <col min="4" max="4" width="10.85546875" style="2" customWidth="1"/>
-    <col min="5" max="5" width="12.42578125" style="3" customWidth="1"/>
-    <col min="6" max="6" width="6.5703125" style="2" hidden="1" customWidth="1"/>
-    <col min="7" max="7" width="10.28515625" style="3" customWidth="1"/>
-    <col min="8" max="8" width="13.7109375" style="3" customWidth="1"/>
-    <col min="9" max="9" width="6.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.7109375" style="3" customWidth="1"/>
-    <col min="11" max="11" width="7.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.88671875" style="2" customWidth="1"/>
+    <col min="5" max="5" width="12.44140625" style="3" customWidth="1"/>
+    <col min="6" max="6" width="6.5546875" style="2" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="10.33203125" style="3" customWidth="1"/>
+    <col min="8" max="8" width="13.6640625" style="3" customWidth="1"/>
+    <col min="9" max="9" width="6.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.6640625" style="3" customWidth="1"/>
+    <col min="11" max="11" width="7.33203125" style="2" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="14" style="3" customWidth="1"/>
-    <col min="13" max="13" width="7.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.5703125" style="3" customWidth="1"/>
-    <col min="15" max="15" width="7.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="7.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.5546875" style="3" customWidth="1"/>
+    <col min="15" max="15" width="7.33203125" style="2" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="11" style="3" customWidth="1"/>
-    <col min="17" max="17" width="7.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="7.33203125" style="2" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="17" style="3" customWidth="1"/>
-    <col min="19" max="19" width="7.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="14.7109375" style="3" customWidth="1"/>
-    <col min="21" max="21" width="7.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="13.7109375" style="3" customWidth="1"/>
-    <col min="23" max="23" width="7.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="13.5703125" style="3" customWidth="1"/>
+    <col min="19" max="19" width="7.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="14.6640625" style="3" customWidth="1"/>
+    <col min="21" max="21" width="7.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="13.6640625" style="3" customWidth="1"/>
+    <col min="23" max="23" width="7.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="13.5546875" style="3" customWidth="1"/>
     <col min="25" max="25" width="7" style="2" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="13.85546875" style="3" customWidth="1"/>
-    <col min="27" max="27" width="7.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="28" max="29" width="9.140625" style="2"/>
-    <col min="30" max="39" width="13.140625" style="2" customWidth="1"/>
-    <col min="40" max="40" width="13.28515625" style="2" customWidth="1"/>
-    <col min="41" max="16384" width="9.140625" style="2"/>
+    <col min="26" max="26" width="13.88671875" style="3" customWidth="1"/>
+    <col min="27" max="27" width="7.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="28" max="29" width="9.109375" style="2"/>
+    <col min="30" max="39" width="13.109375" style="2" customWidth="1"/>
+    <col min="40" max="40" width="13.33203125" style="2" customWidth="1"/>
+    <col min="41" max="16384" width="9.109375" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6200,36 +6214,36 @@
       </c>
       <c r="AA33" s="12"/>
     </row>
-    <row r="34" spans="1:27" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="14"/>
-      <c r="B34" s="14"/>
-      <c r="C34" s="14"/>
-      <c r="D34" s="14"/>
+    <row r="34" spans="1:27" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="13"/>
+      <c r="B34" s="13"/>
+      <c r="C34" s="13"/>
+      <c r="D34" s="13"/>
       <c r="E34" s="13"/>
-      <c r="F34" s="14"/>
+      <c r="F34" s="13"/>
       <c r="G34" s="13"/>
-      <c r="H34" s="14" t="s">
+      <c r="H34" s="13" t="s">
         <v>623</v>
       </c>
-      <c r="I34" s="14"/>
+      <c r="I34" s="13"/>
       <c r="J34" s="13"/>
-      <c r="K34" s="14"/>
+      <c r="K34" s="13"/>
       <c r="L34" s="13"/>
-      <c r="M34" s="14"/>
+      <c r="M34" s="13"/>
       <c r="N34" s="13"/>
-      <c r="O34" s="14"/>
+      <c r="O34" s="13"/>
       <c r="P34" s="13"/>
-      <c r="Q34" s="14"/>
+      <c r="Q34" s="13"/>
       <c r="R34" s="13"/>
-      <c r="S34" s="14"/>
+      <c r="S34" s="13"/>
       <c r="T34" s="13"/>
-      <c r="U34" s="14"/>
+      <c r="U34" s="13"/>
       <c r="V34" s="13"/>
-      <c r="W34" s="14"/>
+      <c r="W34" s="13"/>
       <c r="X34" s="13"/>
-      <c r="Y34" s="14"/>
+      <c r="Y34" s="13"/>
       <c r="Z34" s="13"/>
-      <c r="AA34" s="14"/>
+      <c r="AA34" s="13"/>
     </row>
     <row r="35" spans="1:27" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="14" t="s">
@@ -7574,36 +7588,36 @@
         <v>317</v>
       </c>
     </row>
-    <row r="53" spans="1:27" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="16"/>
-      <c r="B53" s="16"/>
-      <c r="C53" s="16"/>
-      <c r="D53" s="16"/>
+    <row r="53" spans="1:27" s="26" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="15"/>
+      <c r="B53" s="15"/>
+      <c r="C53" s="15"/>
+      <c r="D53" s="15"/>
       <c r="E53" s="15"/>
-      <c r="F53" s="16"/>
+      <c r="F53" s="15"/>
       <c r="G53" s="15"/>
-      <c r="H53" s="16" t="s">
+      <c r="H53" s="15" t="s">
         <v>624</v>
       </c>
-      <c r="I53" s="16"/>
+      <c r="I53" s="15"/>
       <c r="J53" s="15"/>
-      <c r="K53" s="16"/>
+      <c r="K53" s="15"/>
       <c r="L53" s="15"/>
-      <c r="M53" s="16"/>
+      <c r="M53" s="15"/>
       <c r="N53" s="15"/>
-      <c r="O53" s="16"/>
+      <c r="O53" s="15"/>
       <c r="P53" s="15"/>
-      <c r="Q53" s="16"/>
+      <c r="Q53" s="15"/>
       <c r="R53" s="15"/>
-      <c r="S53" s="16"/>
+      <c r="S53" s="15"/>
       <c r="T53" s="15"/>
-      <c r="U53" s="16"/>
+      <c r="U53" s="15"/>
       <c r="V53" s="15"/>
-      <c r="W53" s="16"/>
+      <c r="W53" s="15"/>
       <c r="X53" s="15"/>
-      <c r="Y53" s="16"/>
+      <c r="Y53" s="15"/>
       <c r="Z53" s="15"/>
-      <c r="AA53" s="16"/>
+      <c r="AA53" s="15"/>
     </row>
     <row r="54" spans="1:27" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="16" t="s">
@@ -10106,36 +10120,36 @@
       <c r="AM84" s="6"/>
       <c r="AN84" s="6"/>
     </row>
-    <row r="86" spans="1:40" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="19"/>
-      <c r="B86" s="19"/>
-      <c r="C86" s="19"/>
-      <c r="D86" s="19"/>
+    <row r="86" spans="1:40" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A86" s="20"/>
+      <c r="B86" s="20"/>
+      <c r="C86" s="20"/>
+      <c r="D86" s="20"/>
       <c r="E86" s="20"/>
-      <c r="F86" s="19"/>
+      <c r="F86" s="20"/>
       <c r="G86" s="20"/>
-      <c r="H86" s="19" t="s">
+      <c r="H86" s="20" t="s">
         <v>622</v>
       </c>
-      <c r="I86" s="19"/>
+      <c r="I86" s="20"/>
       <c r="J86" s="20"/>
-      <c r="K86" s="19"/>
+      <c r="K86" s="20"/>
       <c r="L86" s="20"/>
-      <c r="M86" s="19"/>
+      <c r="M86" s="20"/>
       <c r="N86" s="20"/>
-      <c r="O86" s="19"/>
+      <c r="O86" s="20"/>
       <c r="P86" s="20"/>
-      <c r="Q86" s="19"/>
+      <c r="Q86" s="20"/>
       <c r="R86" s="20"/>
-      <c r="S86" s="19"/>
+      <c r="S86" s="20"/>
       <c r="T86" s="20"/>
-      <c r="U86" s="19"/>
+      <c r="U86" s="20"/>
       <c r="V86" s="20"/>
-      <c r="W86" s="19"/>
+      <c r="W86" s="20"/>
       <c r="X86" s="20"/>
-      <c r="Y86" s="19"/>
+      <c r="Y86" s="20"/>
       <c r="Z86" s="20"/>
-      <c r="AA86" s="19"/>
+      <c r="AA86" s="20"/>
     </row>
     <row r="87" spans="1:40" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A87" s="19" t="s">
@@ -10848,26 +10862,17 @@
         <v>800</v>
       </c>
     </row>
-    <row r="97" spans="1:27" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A97" s="21"/>
-      <c r="B97" s="21"/>
-      <c r="C97" s="21"/>
-      <c r="D97" s="21"/>
+    <row r="97" spans="1:27" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A97" s="22"/>
+      <c r="B97" s="22"/>
+      <c r="C97" s="22"/>
+      <c r="D97" s="22"/>
       <c r="E97" s="22"/>
-      <c r="F97" s="21"/>
+      <c r="F97" s="22"/>
       <c r="G97" s="22"/>
-      <c r="H97" s="10" t="s">
+      <c r="H97" s="9" t="s">
         <v>934</v>
       </c>
-      <c r="J97" s="9"/>
-      <c r="L97" s="9"/>
-      <c r="N97" s="9"/>
-      <c r="P97" s="9"/>
-      <c r="R97" s="9"/>
-      <c r="T97" s="9"/>
-      <c r="V97" s="9"/>
-      <c r="X97" s="9"/>
-      <c r="Z97" s="9"/>
     </row>
     <row r="98" spans="1:27" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A98" s="21" t="s">

</xml_diff>

<commit_message>
dbn - 09-04-25 - technician name and mapping changes
</commit_message>
<xml_diff>
--- a/ASCal/mapping.xlsx
+++ b/ASCal/mapping.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1869" uniqueCount="1851">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1872" uniqueCount="1854">
   <si>
     <t>MV1</t>
   </si>
@@ -5581,6 +5581,15 @@
   </si>
   <si>
     <t>calMethod</t>
+  </si>
+  <si>
+    <t>B140</t>
+  </si>
+  <si>
+    <t>Technician Name</t>
+  </si>
+  <si>
+    <t>CurrentUser.Name</t>
   </si>
 </sst>
 </file>
@@ -6388,6 +6397,17 @@
         <v>1850</v>
       </c>
     </row>
+    <row r="33" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="s">
+        <v>1852</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>1851</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>1853</v>
+      </c>
+    </row>
     <row r="34" spans="1:27" s="1" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="23" t="s">
         <v>1445</v>

</xml_diff>